<commit_message>
v2 PCB design complete: audio circuit verified, files committed, parts ordered
Design cloned from v1 in EasyEDA, R3-R6/C3/C4/D1(BAT85)/J7 added and
J6_SWITCH removed. DRC clean; connectivity manually verified from the
exported schematic JSON since EasyEDA Standard has no separate ERC,
which also caught J7's Front L/R pins wired backwards (R3=Right/R4=Left)
-- fixed and re-verified as R3=Left/R4=Right, matching the docs.

Commits the v2 design files (gerbers/bom/easyeda) and retroactively adds
v1's missing schematic JSON export. Adds a new "Audio Addition" tab to
the system BOM for the new parts, now marked ordered. Updates docs across
the repo to reflect Phase 3 status: design done, about to submit to
JLCPCB, firmware (v4.x) not yet started.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/bom/MR2_Reactive_LEDs_System_BOM.xlsx
+++ b/hardware/bom/MR2_Reactive_LEDs_System_BOM.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audio Addition" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1107,4 +1108,268 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16.42578125" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="19.85546875" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Supplier / Source</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Resistor</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>470 Ω Resistor (R3, R4)</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Already on hand</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>RCA channel isolation (Front Left / Front Right) into the audio conditioning circuit</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Bench-validated value; protects source, not used for attenuation</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="42" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Resistor</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>100 kΩ Resistor (R5)</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Already on hand</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Reference-to-ground resistor for the coupling capacitor (C4)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Production-only addition, not part of the validated testing circuit</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Resistor</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>10 kΩ Resistor (R6)</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Already on hand</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Envelope discharge resistor, Node B to GND</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Same role as the testing circuit's R6</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Capacitor</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2.2µF Capacitor (C3)</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Already on hand</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Envelope smoothing capacitor, Node B to GND</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Same role as the testing circuit's C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Capacitor</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Non-polarized Coupling Capacitor (C4)</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Ordered</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>DC-blocking coupling capacitor ahead of the envelope detector</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Must be genuinely non-polarized (ceramic or film, not electrolytic), ~2.2–4.7µF, 16V+ — see docs/audio-reactive-led-plan.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Diode</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BAT85 Schottky Diode (D1)</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Ordered</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Envelope detector rectifying diode</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Production upgrade from the testing circuit's 1N4007 — lower forward voltage improves quiet-passage sensitivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Connectors</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>JST-XH 2.54mm 3-pin Connector (J7)</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Ordered</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>RCA tap input connector (Front Left, Front Right, shield/ground)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Matches the existing J2–J5 connector style already on the board</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>